<commit_message>
Auto-registro SGC: Folio INC-2026-0001
</commit_message>
<xml_diff>
--- a/BD_Reportes_Incoming.xlsx
+++ b/BD_Reportes_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,53 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Dossier_Ruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>INC-2026-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>11:26 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ternium México</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0301682984</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TX6793212</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>/mount/src/incoming-calidad/carpetas_electronicas/INC-2026-0001/Dosier_Calidad_INC-2026-0001.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>